<commit_message>
Demonstrate supply contracts in USD alongside IQD construction
</commit_message>
<xml_diff>
--- a/uploads/01-boq/supply-boq.xlsx
+++ b/uploads/01-boq/supply-boq.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ" sheetId="1" r:id="R947a4d989a144d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ" sheetId="1" r:id="Ra69c641781244547"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -324,7 +324,7 @@
         <x:v>Qty</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>Rate (IQD)</x:v>
+        <x:v>Rate (USD)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
@@ -344,7 +344,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F2" s="7" t="n">
-        <x:v>45000000</x:v>
+        <x:v>34000</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -364,7 +364,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F3" s="10" t="n">
-        <x:v>32000000</x:v>
+        <x:v>24000</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -384,7 +384,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F4" s="7" t="n">
-        <x:v>8500000</x:v>
+        <x:v>6500</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -404,7 +404,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="10" t="n">
-        <x:v>4000000</x:v>
+        <x:v>3000</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -424,7 +424,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="F6" s="7" t="n">
-        <x:v>9000000</x:v>
+        <x:v>7000</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -444,7 +444,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="10" t="n">
-        <x:v>2500000</x:v>
+        <x:v>1900</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>